<commit_message>
Integrated Asset Consolidator into main app
</commit_message>
<xml_diff>
--- a/Master_Asset_Tracker.xlsx
+++ b/Master_Asset_Tracker.xlsx
@@ -515,7 +515,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-17 22:40</t>
+          <t>2026-09-18 21:54</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>

</xml_diff>